<commit_message>
Plan aktualisiert per Excel-Makro
</commit_message>
<xml_diff>
--- a/Trainingsplan.xlsx
+++ b/Trainingsplan.xlsx
@@ -1,23 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326" codeName="{26A90621-87C4-6C01-FD6A-EE6E7C140903}"/>
+  <workbookPr codeName="DieseArbeitsmappe" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\michkern\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\michkern\Desktop\TrainingsplanerPWA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FF0A630-F064-44B9-8A8E-0E37840A4414}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8A34FD55-3AF0-4ADD-BE7A-D60F536C8A8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{516F93C8-1812-4DF3-9B6B-A95E39069BBF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{516F93C8-1812-4DF3-9B6B-A95E39069BBF}"/>
   </bookViews>
   <sheets>
-    <sheet name="Plan_Test" sheetId="2" r:id="rId1"/>
-    <sheet name="Plan1" sheetId="1" r:id="rId2"/>
-    <sheet name="Plan_Test_4" sheetId="3" r:id="rId3"/>
-    <sheet name="Plan_Test_5" sheetId="4" r:id="rId4"/>
+    <sheet name="Upload" sheetId="5" r:id="rId1"/>
+    <sheet name="PlanMichiHome" sheetId="6" r:id="rId2"/>
+    <sheet name="Plan_Test" sheetId="2" r:id="rId3"/>
+    <sheet name="Plan1" sheetId="1" r:id="rId4"/>
+    <sheet name="Plan_Test_4" sheetId="3" r:id="rId5"/>
+    <sheet name="Plan_Test_5" sheetId="4" r:id="rId6"/>
   </sheets>
+  <functionGroups builtInGroupCount="19"/>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -42,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="25">
   <si>
     <t>Laufen</t>
   </si>
@@ -96,6 +99,32 @@
   </si>
   <si>
     <t>dddddd</t>
+  </si>
+  <si>
+    <t>Seilspringen</t>
+  </si>
+  <si>
+    <t>Keine</t>
+  </si>
+  <si>
+    <t>Boden</t>
+  </si>
+  <si>
+    <t>1. 50 Liegestütz
+2. 50 Situps
+3. 45s Bauchroller (ca. 10 Wiederholungen)</t>
+  </si>
+  <si>
+    <t>Sandsack</t>
+  </si>
+  <si>
+    <t>Sandsack komplett</t>
+  </si>
+  <si>
+    <t>Schattenboxen mit Gewichte</t>
+  </si>
+  <si>
+    <t>Sandsack nur Beine</t>
   </si>
 </sst>
 </file>
@@ -167,6 +196,83 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/ctrlProps/ctrlProp1.xml><?xml version="1.0" encoding="utf-8"?>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Button" lockText="1"/>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor>
+        <xdr:from>
+          <xdr:col>1</xdr:col>
+          <xdr:colOff>123825</xdr:colOff>
+          <xdr:row>1</xdr:row>
+          <xdr:rowOff>142875</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>5</xdr:col>
+          <xdr:colOff>38100</xdr:colOff>
+          <xdr:row>5</xdr:row>
+          <xdr:rowOff>85725</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="5121" name="Button 1" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s5121"/>
+                </a:ext>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000001140000}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:ln w="9525">
+              <a:miter lim="800000"/>
+              <a:headEnd/>
+              <a:tailEnd/>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" wrap="square" lIns="27432" tIns="27432" rIns="27432" bIns="27432" anchor="ctr" upright="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr algn="ctr" rtl="0">
+                <a:defRPr sz="1000"/>
+              </a:pPr>
+              <a:r>
+                <a:rPr lang="de-DE" sz="1100" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                  <a:solidFill>
+                    <a:srgbClr val="000000"/>
+                  </a:solidFill>
+                  <a:latin typeface="Aptos Narrow"/>
+                </a:rPr>
+                <a:t>Upload</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+        <xdr:clientData fPrintsWithSheet="0"/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -485,7 +591,303 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDC923CF-6441-4B69-8F08-DD20C5A223E6}">
+  <sheetPr codeName="Tabelle5"/>
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x14">
+      <controls>
+        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+          <mc:Choice Requires="x14">
+            <control shapeId="5121" r:id="rId3" name="Button 1">
+              <controlPr defaultSize="0" print="0" autoFill="0" autoPict="0" macro="[0]!UploadToGitHub">
+                <anchor moveWithCells="1" sizeWithCells="1">
+                  <from>
+                    <xdr:col>1</xdr:col>
+                    <xdr:colOff>123825</xdr:colOff>
+                    <xdr:row>1</xdr:row>
+                    <xdr:rowOff>142875</xdr:rowOff>
+                  </from>
+                  <to>
+                    <xdr:col>5</xdr:col>
+                    <xdr:colOff>38100</xdr:colOff>
+                    <xdr:row>5</xdr:row>
+                    <xdr:rowOff>85725</xdr:rowOff>
+                  </to>
+                </anchor>
+              </controlPr>
+            </control>
+          </mc:Choice>
+        </mc:AlternateContent>
+      </controls>
+    </mc:Choice>
+  </mc:AlternateContent>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8466D9D2-2DE6-4350-85C3-330F2B19D1C9}">
+  <sheetPr codeName="Tabelle6"/>
+  <dimension ref="A2:F15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="25.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="56.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="1">
+        <v>7</v>
+      </c>
+      <c r="C3" s="1">
+        <v>1</v>
+      </c>
+      <c r="D3" s="1">
+        <v>0.8</v>
+      </c>
+      <c r="E3" s="1">
+        <f>(B3*C3)+(D3*C3)</f>
+        <v>7.8</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="1">
+        <v>3.2</v>
+      </c>
+      <c r="C4" s="1">
+        <v>1</v>
+      </c>
+      <c r="D4" s="1">
+        <v>1</v>
+      </c>
+      <c r="E4" s="1">
+        <f>(B4*C4)+(D4*C4)</f>
+        <v>4.2</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" s="1">
+        <v>3</v>
+      </c>
+      <c r="C5" s="1">
+        <v>1</v>
+      </c>
+      <c r="D5" s="1">
+        <v>0.8</v>
+      </c>
+      <c r="E5" s="1">
+        <f>(B5*C5)+(D5*C5)</f>
+        <v>3.8</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" s="1">
+        <v>3.2</v>
+      </c>
+      <c r="C6" s="1">
+        <v>1</v>
+      </c>
+      <c r="D6" s="1">
+        <v>1</v>
+      </c>
+      <c r="E6" s="1">
+        <f>(B6*C6)+(D6*C6)</f>
+        <v>4.2</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="1">
+        <v>3</v>
+      </c>
+      <c r="C7" s="1">
+        <v>1</v>
+      </c>
+      <c r="D7" s="1">
+        <v>0.8</v>
+      </c>
+      <c r="E7" s="1">
+        <f>(B7*C7)+(D7*C7)</f>
+        <v>3.8</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" s="1">
+        <v>3.2</v>
+      </c>
+      <c r="C8" s="1">
+        <v>1</v>
+      </c>
+      <c r="D8" s="1">
+        <v>1</v>
+      </c>
+      <c r="E8" s="1">
+        <f>(B8*C8)+(D8*C8)</f>
+        <v>4.2</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B9" s="1">
+        <v>3</v>
+      </c>
+      <c r="C9" s="1">
+        <v>1</v>
+      </c>
+      <c r="D9" s="1">
+        <v>0.8</v>
+      </c>
+      <c r="E9" s="1">
+        <f>(B9*C9)+(D9*C9)</f>
+        <v>3.8</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" s="1">
+        <v>3.2</v>
+      </c>
+      <c r="C10" s="1">
+        <v>1</v>
+      </c>
+      <c r="D10" s="1">
+        <v>1</v>
+      </c>
+      <c r="E10" s="1">
+        <f>(B10*C10)+(D10*C10)</f>
+        <v>4.2</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11" s="1">
+        <v>3</v>
+      </c>
+      <c r="C11" s="1">
+        <v>1</v>
+      </c>
+      <c r="D11" s="1">
+        <v>0.8</v>
+      </c>
+      <c r="E11" s="1">
+        <f>(B11*C11)+(D11*C11)</f>
+        <v>3.8</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" s="1">
+        <v>3.2</v>
+      </c>
+      <c r="C12" s="1">
+        <v>1</v>
+      </c>
+      <c r="D12" s="1">
+        <v>1</v>
+      </c>
+      <c r="E12" s="1">
+        <f>(B12*C12)+(D12*C12)</f>
+        <v>4.2</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D15" t="s">
+        <v>14</v>
+      </c>
+      <c r="E15">
+        <f>SUM(E3:E12)</f>
+        <v>44</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79EC839E-A5A5-4649-B708-16C9527B953B}">
+  <sheetPr codeName="Tabelle1"/>
   <dimension ref="A2:F10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -633,8 +1035,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{424A7408-8884-4222-B545-A3B808670452}">
+  <sheetPr codeName="Tabelle2"/>
   <dimension ref="A2:F10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -782,8 +1185,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F38893D4-C661-4283-A65E-F50E2E2C3791}">
+  <sheetPr codeName="Tabelle3"/>
   <dimension ref="A2:F12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -973,8 +1377,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F18A1C6-F7D4-457B-8570-998CF178D384}">
+  <sheetPr codeName="Tabelle4"/>
   <dimension ref="A2:F12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>

</xml_diff>

<commit_message>
Plan synchronisiert & aktualisiert per Excel-Makro
</commit_message>
<xml_diff>
--- a/Trainingsplan.xlsx
+++ b/Trainingsplan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\michkern\Desktop\TrainingsplanerPWA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3DC862DC-9E04-473F-94EA-17594153B904}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5282AB7B-24D4-429D-B6FF-CCE8DDA3C286}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{516F93C8-1812-4DF3-9B6B-A95E39069BBF}"/>
   </bookViews>
@@ -19,6 +19,7 @@
     <sheet name="Plan1" sheetId="1" r:id="rId4"/>
     <sheet name="Plan_Test_4" sheetId="3" r:id="rId5"/>
     <sheet name="Plan_Test_5" sheetId="4" r:id="rId6"/>
+    <sheet name="PlanMichiHome (2)" sheetId="7" r:id="rId7"/>
   </sheets>
   <functionGroups builtInGroupCount="19"/>
   <calcPr calcId="191029"/>
@@ -45,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="25">
   <si>
     <t>Laufen</t>
   </si>
@@ -131,13 +132,19 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -605,7 +612,7 @@
         <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
           <mc:Choice Requires="x14">
             <control shapeId="5121" r:id="rId3" name="Button 1">
-              <controlPr defaultSize="0" print="0" autoFill="0" autoPict="0" macro="[0]!UploadToGitHub">
+              <controlPr defaultSize="0" print="0" autoFill="0" autoPict="0" macro="[0]!SyncAndUploadToGitHub">
                 <anchor moveWithCells="1" sizeWithCells="1">
                   <from>
                     <xdr:col>1</xdr:col>
@@ -675,7 +682,7 @@
         <v>0.8</v>
       </c>
       <c r="E3" s="1">
-        <f>(B3*C3)+(D3*C3)</f>
+        <f t="shared" ref="E3:E12" si="0">(B3*C3)+(D3*C3)</f>
         <v>7.8</v>
       </c>
       <c r="F3" s="2" t="s">
@@ -696,7 +703,7 @@
         <v>1</v>
       </c>
       <c r="E4" s="1">
-        <f>(B4*C4)+(D4*C4)</f>
+        <f t="shared" si="0"/>
         <v>4.2</v>
       </c>
       <c r="F4" s="2" t="s">
@@ -717,7 +724,7 @@
         <v>0.8</v>
       </c>
       <c r="E5" s="1">
-        <f>(B5*C5)+(D5*C5)</f>
+        <f t="shared" si="0"/>
         <v>3.8</v>
       </c>
       <c r="F5" s="2" t="s">
@@ -738,7 +745,7 @@
         <v>1</v>
       </c>
       <c r="E6" s="1">
-        <f>(B6*C6)+(D6*C6)</f>
+        <f t="shared" si="0"/>
         <v>4.2</v>
       </c>
       <c r="F6" s="2" t="s">
@@ -759,7 +766,7 @@
         <v>0.8</v>
       </c>
       <c r="E7" s="1">
-        <f>(B7*C7)+(D7*C7)</f>
+        <f t="shared" si="0"/>
         <v>3.8</v>
       </c>
       <c r="F7" s="2" t="s">
@@ -780,7 +787,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="1">
-        <f>(B8*C8)+(D8*C8)</f>
+        <f t="shared" si="0"/>
         <v>4.2</v>
       </c>
       <c r="F8" s="2" t="s">
@@ -801,7 +808,7 @@
         <v>0.8</v>
       </c>
       <c r="E9" s="1">
-        <f>(B9*C9)+(D9*C9)</f>
+        <f t="shared" si="0"/>
         <v>3.8</v>
       </c>
       <c r="F9" s="2" t="s">
@@ -822,7 +829,7 @@
         <v>1</v>
       </c>
       <c r="E10" s="1">
-        <f>(B10*C10)+(D10*C10)</f>
+        <f t="shared" si="0"/>
         <v>4.2</v>
       </c>
       <c r="F10" s="2" t="s">
@@ -843,7 +850,7 @@
         <v>0.8</v>
       </c>
       <c r="E11" s="1">
-        <f>(B11*C11)+(D11*C11)</f>
+        <f t="shared" si="0"/>
         <v>3.8</v>
       </c>
       <c r="F11" s="2" t="s">
@@ -864,7 +871,7 @@
         <v>1</v>
       </c>
       <c r="E12" s="1">
-        <f>(B12*C12)+(D12*C12)</f>
+        <f t="shared" si="0"/>
         <v>4.2</v>
       </c>
       <c r="F12" s="2" t="s">
@@ -1567,4 +1574,259 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{526DC257-88C4-4D20-A37D-1F8D303F1381}">
+  <sheetPr codeName="Tabelle7"/>
+  <dimension ref="A2:F15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="25.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="56.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="1">
+        <v>7</v>
+      </c>
+      <c r="C3" s="1">
+        <v>1</v>
+      </c>
+      <c r="D3" s="1">
+        <v>0.8</v>
+      </c>
+      <c r="E3" s="1">
+        <f t="shared" ref="E3:E12" si="0">(B3*C3)+(D3*C3)</f>
+        <v>7.8</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="1">
+        <v>3.2</v>
+      </c>
+      <c r="C4" s="1">
+        <v>1</v>
+      </c>
+      <c r="D4" s="1">
+        <v>1</v>
+      </c>
+      <c r="E4" s="1">
+        <f t="shared" si="0"/>
+        <v>4.2</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" s="1">
+        <v>3</v>
+      </c>
+      <c r="C5" s="1">
+        <v>1</v>
+      </c>
+      <c r="D5" s="1">
+        <v>0.8</v>
+      </c>
+      <c r="E5" s="1">
+        <f t="shared" si="0"/>
+        <v>3.8</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" s="1">
+        <v>3.2</v>
+      </c>
+      <c r="C6" s="1">
+        <v>1</v>
+      </c>
+      <c r="D6" s="1">
+        <v>1</v>
+      </c>
+      <c r="E6" s="1">
+        <f t="shared" si="0"/>
+        <v>4.2</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="1">
+        <v>3</v>
+      </c>
+      <c r="C7" s="1">
+        <v>1</v>
+      </c>
+      <c r="D7" s="1">
+        <v>0.8</v>
+      </c>
+      <c r="E7" s="1">
+        <f t="shared" si="0"/>
+        <v>3.8</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" s="1">
+        <v>3.2</v>
+      </c>
+      <c r="C8" s="1">
+        <v>1</v>
+      </c>
+      <c r="D8" s="1">
+        <v>1</v>
+      </c>
+      <c r="E8" s="1">
+        <f t="shared" si="0"/>
+        <v>4.2</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B9" s="1">
+        <v>3</v>
+      </c>
+      <c r="C9" s="1">
+        <v>1</v>
+      </c>
+      <c r="D9" s="1">
+        <v>0.8</v>
+      </c>
+      <c r="E9" s="1">
+        <f t="shared" si="0"/>
+        <v>3.8</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" s="1">
+        <v>3.2</v>
+      </c>
+      <c r="C10" s="1">
+        <v>1</v>
+      </c>
+      <c r="D10" s="1">
+        <v>1</v>
+      </c>
+      <c r="E10" s="1">
+        <f t="shared" si="0"/>
+        <v>4.2</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11" s="1">
+        <v>3</v>
+      </c>
+      <c r="C11" s="1">
+        <v>1</v>
+      </c>
+      <c r="D11" s="1">
+        <v>0.8</v>
+      </c>
+      <c r="E11" s="1">
+        <f t="shared" si="0"/>
+        <v>3.8</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" s="1">
+        <v>3.2</v>
+      </c>
+      <c r="C12" s="1">
+        <v>1</v>
+      </c>
+      <c r="D12" s="1">
+        <v>1</v>
+      </c>
+      <c r="E12" s="1">
+        <f t="shared" si="0"/>
+        <v>4.2</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D15" t="s">
+        <v>14</v>
+      </c>
+      <c r="E15">
+        <f>SUM(E3:E12)</f>
+        <v>44</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>